<commit_message>
Save library recording Amazon learning - c5056382-69db-48cd-942e-6e184d2599c8 - 2026-10-13T13:07:40.448937Z
</commit_message>
<xml_diff>
--- a/library/projects/qa-sample-app/recordings/c5056382-69db-48cd-942e-6e184d2599c8/resources/azure-devops.xlsx
+++ b/library/projects/qa-sample-app/recordings/c5056382-69db-48cd-942e-6e184d2599c8/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,6 +445,92 @@
       <c r="F1" t="inlineStr">
         <is>
           <t>Screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Amazon learning</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://www.amazon.com/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Amazon learning</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click Click the button below to continue shopping
+Continue shopping
+Conditions of Use</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "body:nth-of-type(1) &gt; div:nth-of-type(1)", "x": 706, "y": 266, "text": "Click the button below to continue shopping\nContinue shopping\nConditions of Use ", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Amazon learning</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Click Continue shopping</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "form:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; span:nth-of-type(1) &gt; span:nth-of-type(1) &gt; button:nth-of-type(1)", "x": 568, "y": 213, "text": "Continue shopping", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
         </is>
       </c>
     </row>

</xml_diff>